<commit_message>
Polish weather API report portfolio project
</commit_message>
<xml_diff>
--- a/projects/03_api_report_tool/output/weather_report.xlsx
+++ b/projects/03_api_report_tool/output/weather_report.xlsx
@@ -7,10 +7,17 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="current_weather" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="daily_forecast" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="report_summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="current_weather" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="daily_forecast" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="api_errors" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'report_summary'!$A$1:$B$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'current_weather'!$A$1:$H$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'daily_forecast'!$A$1:$E$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'api_errors'!$A$1:$E$1</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -18,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,13 +33,22 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -47,8 +63,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -123,6 +142,48 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ReportSummaryTable" displayName="ReportSummaryTable" ref="A1:B6" headerRowCount="1">
+  <autoFilter ref="A1:B6"/>
+  <tableColumns count="2">
+    <tableColumn id="1" name="metric"/>
+    <tableColumn id="2" name="value"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CurrentWeatherTable" displayName="CurrentWeatherTable" ref="A1:H4" headerRowCount="1">
+  <autoFilter ref="A1:H4"/>
+  <tableColumns count="8">
+    <tableColumn id="1" name="city"/>
+    <tableColumn id="2" name="time"/>
+    <tableColumn id="3" name="temperature"/>
+    <tableColumn id="4" name="temperature_unit"/>
+    <tableColumn id="5" name="humidity"/>
+    <tableColumn id="6" name="humidity_unit"/>
+    <tableColumn id="7" name="wind_speed"/>
+    <tableColumn id="8" name="wind_speed_unit"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="DailyForecastTable" displayName="DailyForecastTable" ref="A1:E10" headerRowCount="1">
+  <autoFilter ref="A1:E10"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="city"/>
+    <tableColumn id="2" name="date"/>
+    <tableColumn id="3" name="temperature_max"/>
+    <tableColumn id="4" name="temperature_min"/>
+    <tableColumn id="5" name="precipitation_sum"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -414,161 +475,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>city</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>time</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>temperature</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>temperature_unit</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>humidity</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>humidity_unit</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>wind_speed</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>wind_speed_unit</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Shanghai</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>2026-05-17T23:00</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>°C</t>
-        </is>
-      </c>
-      <c r="E2" t="n">
-        <v>81</v>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>15.3</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>km/h</t>
-        </is>
+          <t>Configured cities</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Beijing</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>2026-05-17T23:00</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>18</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>°C</t>
-        </is>
-      </c>
-      <c r="E3" t="n">
-        <v>95</v>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>9.1</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>km/h</t>
-        </is>
+          <t>Successful cities</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>New York</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>2026-05-17T11:00</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>°C</t>
-        </is>
-      </c>
-      <c r="E4" t="n">
-        <v>42</v>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>km/h</t>
-        </is>
+          <t>Failed cities</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Current weather rows</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Forecast rows</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>9</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:B6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -578,31 +559,216 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>temperature</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>temperature_unit</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>humidity</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>humidity_unit</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>wind_speed</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>wind_speed_unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Shanghai</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-05-24T10:45</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>87</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>km/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Beijing</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2026-05-24T10:45</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>25.5</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>73</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>km/h</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>New York</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2026-05-23T22:45</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>°C</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>87</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>km/h</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>city</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>temperature_max</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>temperature_min</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>precipitation_sum</t>
         </is>
@@ -616,17 +782,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>29.6</v>
+        <v>27.8</v>
       </c>
       <c r="D2" t="n">
-        <v>19.3</v>
+        <v>22.6</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="3">
@@ -637,17 +803,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>28.7</v>
+        <v>32.6</v>
       </c>
       <c r="D3" t="n">
-        <v>19.8</v>
+        <v>23.6</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="4">
@@ -658,17 +824,17 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>28.7</v>
+        <v>28</v>
       </c>
       <c r="D4" t="n">
-        <v>20.5</v>
+        <v>24.9</v>
       </c>
       <c r="E4" t="n">
-        <v>6.3</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="5">
@@ -679,17 +845,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20.3</v>
+        <v>28.5</v>
       </c>
       <c r="D5" t="n">
-        <v>17.6</v>
+        <v>18.9</v>
       </c>
       <c r="E5" t="n">
-        <v>48.5</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="6">
@@ -700,17 +866,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>26.5</v>
+        <v>21.6</v>
       </c>
       <c r="D6" t="n">
-        <v>17.5</v>
+        <v>18.5</v>
       </c>
       <c r="E6" t="n">
-        <v>7.8</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="7">
@@ -721,14 +887,14 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25.4</v>
+        <v>26.6</v>
       </c>
       <c r="D7" t="n">
-        <v>17.1</v>
+        <v>17.8</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -742,17 +908,17 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2026-05-17</t>
+          <t>2026-05-23</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>31.4</v>
+        <v>13.6</v>
       </c>
       <c r="D8" t="n">
-        <v>18.3</v>
+        <v>9.6</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>9.800000000000001</v>
       </c>
     </row>
     <row r="9">
@@ -763,17 +929,17 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-24</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>31.2</v>
+        <v>13.6</v>
       </c>
       <c r="D9" t="n">
-        <v>17.1</v>
+        <v>10</v>
       </c>
       <c r="E9" t="n">
-        <v>0</v>
+        <v>11.52</v>
       </c>
     </row>
     <row r="10">
@@ -784,20 +950,73 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>30.9</v>
+        <v>24.2</v>
       </c>
       <c r="D10" t="n">
-        <v>16.8</v>
+        <v>13.6</v>
       </c>
       <c r="E10" t="n">
-        <v>0</v>
+        <v>2.2</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>city</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>latitude</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>longitude</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>attempts</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>